<commit_message>
Updated wording of iac automation gui
</commit_message>
<xml_diff>
--- a/EnergyCharts/EnergyCharts.xlsx
+++ b/EnergyCharts/EnergyCharts.xlsx
@@ -1,30 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexr\iac_work\IAC-Automation-GUI\EnergyCharts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82629BF0-67B3-472A-B02D-B23A41F40F38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF3E307C-BF75-4ED0-BD49-6E86CAC2C5A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="338" yWindow="2250" windowWidth="18839" windowHeight="11183" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="3" r:id="rId1"/>
-    <sheet name="Water Bill" sheetId="17" r:id="rId2"/>
-    <sheet name="Monthly Charts" sheetId="12" r:id="rId3"/>
-    <sheet name="Total Energy" sheetId="5" r:id="rId4"/>
-    <sheet name="Monthly Cost" sheetId="16" r:id="rId5"/>
+    <sheet name="Monthly Charts" sheetId="12" r:id="rId2"/>
+    <sheet name="Total Energy" sheetId="5" r:id="rId3"/>
+    <sheet name="Monthly Cost" sheetId="16" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw Data'!$K$1:$N$19</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Monthly Charts'!$A$1:$R$51</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Monthly Cost'!$G$1:$M$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Monthly Charts'!$A$1:$R$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Monthly Cost'!$G$1:$M$19</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Raw Data'!$A$1:$O$25</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Total Energy'!$F$1:$K$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Total Energy'!$F$1:$K$27</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,8 +42,35 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={83BABB99-64A9-4C76-931E-7394AAFD09FD}</author>
+    <author>tc={D1BC6906-84CA-4A7C-902B-5F76AE15F688}</author>
+  </authors>
+  <commentList>
+    <comment ref="C7" authorId="0" shapeId="0" xr:uid="{83BABB99-64A9-4C76-931E-7394AAFD09FD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Values being added from account numbers in order:  (501-00) + (501-06) + (502-09)</t>
+      </text>
+    </comment>
+    <comment ref="L7" authorId="1" shapeId="0" xr:uid="{D1BC6906-84CA-4A7C-902B-5F76AE15F688}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Values being added from account numbers in order:  (501-00) + (948-03) + (460-18) + (50-303) + (3-4959) + (17427) + (3-4958) + (42923) + (3-4898)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="51">
   <si>
     <t>Electricity</t>
   </si>
@@ -210,50 +236,12 @@
   <si>
     <t>Start Month:</t>
   </si>
-  <si>
-    <t>Water In</t>
-  </si>
-  <si>
-    <t>Price</t>
-  </si>
-  <si>
-    <t>Effluent Out</t>
-  </si>
-  <si>
-    <t>Total Price</t>
-  </si>
-  <si>
-    <t>Gal</t>
-  </si>
-  <si>
-    <t>$</t>
-  </si>
-  <si>
-    <t>Unit Price</t>
-  </si>
-  <si>
-    <t>$/gal</t>
-  </si>
-  <si>
-    <t>Jan 24 - Mar 24</t>
-  </si>
-  <si>
-    <t>Apr 24 - Jun 24</t>
-  </si>
-  <si>
-    <t>Jul 24 - Sept 24</t>
-  </si>
-  <si>
-    <t>Oct 23- Dec 23</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="13">
-    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
-    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
+  <numFmts count="9">
     <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -263,10 +251,8 @@
     <numFmt numFmtId="167" formatCode="mm/dd/yy"/>
     <numFmt numFmtId="168" formatCode="mmm\ yy"/>
     <numFmt numFmtId="169" formatCode="[$-409]mmm\ yyyy;@"/>
-    <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.000_);[Red]\(&quot;$&quot;#,##0.000\)"/>
-    <numFmt numFmtId="171" formatCode="&quot;$&quot;#,##0.0000_);[Red]\(&quot;$&quot;#,##0.0000\)"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -364,39 +350,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -427,14 +382,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="43">
+  <borders count="33">
     <border>
       <left/>
       <right/>
@@ -842,162 +791,12 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thick">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thick">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="139">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1275,64 +1074,6 @@
     <xf numFmtId="37" fontId="5" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="17" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="6" fontId="17" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="6" fontId="17" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="16" fontId="17" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="17" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="6" fontId="17" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="6" fontId="17" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="8" fontId="17" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="37" fontId="5" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="170" fontId="17" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="171" fontId="17" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1772,40 +1513,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>Oct 23</c:v>
+                  <c:v>Jan 24</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Nov 23</c:v>
+                  <c:v>Feb 24</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Dec 23</c:v>
+                  <c:v>Mar 24</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Jan 24</c:v>
+                  <c:v>Apr 24</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Feb 24</c:v>
+                  <c:v>May 24</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Mar 24</c:v>
+                  <c:v>Jun 24</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Apr 24</c:v>
+                  <c:v>Jul 24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>May 24</c:v>
+                  <c:v>Aug 24</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Jun 24</c:v>
+                  <c:v>Sep 24</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Jul 24</c:v>
+                  <c:v>Oct 24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Aug 24</c:v>
+                  <c:v>Nov 24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sep 24</c:v>
+                  <c:v>Dec 24</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1817,40 +1558,40 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>4981000</c:v>
+                  <c:v>924821</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4992000</c:v>
+                  <c:v>824553</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5972000</c:v>
+                  <c:v>866265</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>6395000</c:v>
+                  <c:v>1043239</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5348000</c:v>
+                  <c:v>1004442</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5675000</c:v>
+                  <c:v>1175894</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>5840000</c:v>
+                  <c:v>1283358</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>5039000</c:v>
+                  <c:v>1189529</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>5326000</c:v>
+                  <c:v>1103782</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>5886000</c:v>
+                  <c:v>1000871</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>5572000</c:v>
+                  <c:v>972150</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>5217000</c:v>
+                  <c:v>973189</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2241,40 +1982,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>Oct 23</c:v>
+                  <c:v>Jan 24</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Nov 23</c:v>
+                  <c:v>Feb 24</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Dec 23</c:v>
+                  <c:v>Mar 24</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Jan 24</c:v>
+                  <c:v>Apr 24</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Feb 24</c:v>
+                  <c:v>May 24</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Mar 24</c:v>
+                  <c:v>Jun 24</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Apr 24</c:v>
+                  <c:v>Jul 24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>May 24</c:v>
+                  <c:v>Aug 24</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Jun 24</c:v>
+                  <c:v>Sep 24</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Jul 24</c:v>
+                  <c:v>Oct 24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Aug 24</c:v>
+                  <c:v>Nov 24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sep 24</c:v>
+                  <c:v>Dec 24</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2286,40 +2027,40 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>11081</c:v>
+                  <c:v>1511.9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>10200</c:v>
+                  <c:v>1587.6999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10744</c:v>
+                  <c:v>1794.1</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>10744</c:v>
+                  <c:v>1878.8999999999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>11184</c:v>
+                  <c:v>1960</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>11042</c:v>
+                  <c:v>2239.1</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>11042</c:v>
+                  <c:v>2394</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>10588</c:v>
+                  <c:v>2411.8000000000002</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>11094</c:v>
+                  <c:v>2221.6</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>12299</c:v>
+                  <c:v>1928.1000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>12390</c:v>
+                  <c:v>2103.8000000000002</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>11340</c:v>
+                  <c:v>1725.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2700,40 +2441,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>Oct 23</c:v>
+                  <c:v>Jan 24</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Nov 23</c:v>
+                  <c:v>Feb 24</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Dec 23</c:v>
+                  <c:v>Mar 24</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Jan 24</c:v>
+                  <c:v>Apr 24</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Feb 24</c:v>
+                  <c:v>May 24</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Mar 24</c:v>
+                  <c:v>Jun 24</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Apr 24</c:v>
+                  <c:v>Jul 24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>May 24</c:v>
+                  <c:v>Aug 24</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Jun 24</c:v>
+                  <c:v>Sep 24</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Jul 24</c:v>
+                  <c:v>Oct 24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Aug 24</c:v>
+                  <c:v>Nov 24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sep 24</c:v>
+                  <c:v>Dec 24</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2745,40 +2486,40 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>12036.040799999999</c:v>
+                  <c:v>19356.980099999997</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>25294.250800000002</c:v>
+                  <c:v>17571.233899999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>28236.698</c:v>
+                  <c:v>18373.1355</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>37686.364800000003</c:v>
+                  <c:v>17373.641</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>30949.049599999998</c:v>
+                  <c:v>16282.555400000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>26336.984799999998</c:v>
+                  <c:v>15154.398999999999</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>17759.008400000002</c:v>
+                  <c:v>15527.440499999997</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7370.6220000000003</c:v>
+                  <c:v>16815.338100000001</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4192.692</c:v>
+                  <c:v>17420.905800000004</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3046.5652</c:v>
+                  <c:v>18208.920900000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3515.3552</c:v>
+                  <c:v>20512.359899999999</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>5362.4396000000006</c:v>
+                  <c:v>9807.3008000000009</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3155,40 +2896,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>Oct 23</c:v>
+                  <c:v>Jan 24</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Nov 23</c:v>
+                  <c:v>Feb 24</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Dec 23</c:v>
+                  <c:v>Mar 24</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Jan 24</c:v>
+                  <c:v>Apr 24</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Feb 24</c:v>
+                  <c:v>May 24</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Mar 24</c:v>
+                  <c:v>Jun 24</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Apr 24</c:v>
+                  <c:v>Jul 24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>May 24</c:v>
+                  <c:v>Aug 24</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Jun 24</c:v>
+                  <c:v>Sep 24</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Jul 24</c:v>
+                  <c:v>Oct 24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Aug 24</c:v>
+                  <c:v>Nov 24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sep 24</c:v>
+                  <c:v>Dec 24</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3200,40 +2941,40 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>336267.31</c:v>
+                  <c:v>106397.86</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>337009.91999999998</c:v>
+                  <c:v>95101.49</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>403169.72</c:v>
+                  <c:v>100800.73</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>431726.45</c:v>
+                  <c:v>121946.65</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>361043.48</c:v>
+                  <c:v>117553.12999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>383119.25</c:v>
+                  <c:v>137534.25</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>394258.4</c:v>
+                  <c:v>151332.35</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>340182.89</c:v>
+                  <c:v>141123.71</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>359558.26</c:v>
+                  <c:v>131091.88999999998</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>397363.86</c:v>
+                  <c:v>119489.42</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>376165.72</c:v>
+                  <c:v>115818.54000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>352199.67</c:v>
+                  <c:v>116031.34</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3626,40 +3367,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>Oct 23</c:v>
+                  <c:v>Jan 24</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Nov 23</c:v>
+                  <c:v>Feb 24</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Dec 23</c:v>
+                  <c:v>Mar 24</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Jan 24</c:v>
+                  <c:v>Apr 24</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Feb 24</c:v>
+                  <c:v>May 24</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Mar 24</c:v>
+                  <c:v>Jun 24</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Apr 24</c:v>
+                  <c:v>Jul 24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>May 24</c:v>
+                  <c:v>Aug 24</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Jun 24</c:v>
+                  <c:v>Sep 24</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Jul 24</c:v>
+                  <c:v>Oct 24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Aug 24</c:v>
+                  <c:v>Nov 24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sep 24</c:v>
+                  <c:v>Dec 24</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -3671,40 +3412,40 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>17843.61</c:v>
+                  <c:v>3727.2400000000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17843.61</c:v>
+                  <c:v>3654.9300000000003</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20304.8</c:v>
+                  <c:v>4105.5200000000004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>21535.39</c:v>
+                  <c:v>4318.84</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>17228.310000000001</c:v>
+                  <c:v>4585.8</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>18458.91</c:v>
+                  <c:v>26620.42</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>19689.5</c:v>
+                  <c:v>29423.26</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>17843.61</c:v>
+                  <c:v>29498.550000000003</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>18271.48</c:v>
+                  <c:v>26660.23</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>19189.689999999999</c:v>
+                  <c:v>4596.1099999999997</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>17390.66</c:v>
+                  <c:v>6038.83</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>17990.34</c:v>
+                  <c:v>5131.53</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4081,40 +3822,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>Oct 23</c:v>
+                  <c:v>Jan 24</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Nov 23</c:v>
+                  <c:v>Feb 24</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Dec 23</c:v>
+                  <c:v>Mar 24</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Jan 24</c:v>
+                  <c:v>Apr 24</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Feb 24</c:v>
+                  <c:v>May 24</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Mar 24</c:v>
+                  <c:v>Jun 24</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Apr 24</c:v>
+                  <c:v>Jul 24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>May 24</c:v>
+                  <c:v>Aug 24</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Jun 24</c:v>
+                  <c:v>Sep 24</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Jul 24</c:v>
+                  <c:v>Oct 24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Aug 24</c:v>
+                  <c:v>Nov 24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sep 24</c:v>
+                  <c:v>Dec 24</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -4126,40 +3867,40 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>49724.82</c:v>
+                  <c:v>87857.74</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13191.5</c:v>
+                  <c:v>65523.329999999994</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>43547.51</c:v>
+                  <c:v>66562.8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>251777.42</c:v>
+                  <c:v>52165.7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>58848.990000000005</c:v>
+                  <c:v>49743.42</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-3183.3199999999997</c:v>
+                  <c:v>46165.399999999994</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>61041.850000000006</c:v>
+                  <c:v>48984.39</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>42994.85</c:v>
+                  <c:v>50635.75</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>37352.270000000004</c:v>
+                  <c:v>51575.020000000004</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>35079.659999999996</c:v>
+                  <c:v>53352.630000000005</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>34223.160000000003</c:v>
+                  <c:v>75418.23</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>37024.480000000003</c:v>
+                  <c:v>27233.280000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4572,13 +4313,8 @@
                   <a:pPr>
                     <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                       <a:solidFill>
-                        <a:schemeClr val="bg1"/>
+                        <a:schemeClr val="accent5"/>
                       </a:solidFill>
-                      <a:effectLst>
-                        <a:glow rad="76200">
-                          <a:schemeClr val="tx1"/>
-                        </a:glow>
-                      </a:effectLst>
                       <a:latin typeface="+mn-lt"/>
                       <a:ea typeface="+mn-ea"/>
                       <a:cs typeface="+mn-cs"/>
@@ -4587,7 +4323,7 @@
                   <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
-              <c:dLblPos val="bestFit"/>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="1"/>
@@ -4620,13 +4356,8 @@
                   <a:pPr>
                     <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                       <a:solidFill>
-                        <a:schemeClr val="bg1"/>
+                        <a:schemeClr val="accent6"/>
                       </a:solidFill>
-                      <a:effectLst>
-                        <a:glow rad="76200">
-                          <a:schemeClr val="tx1"/>
-                        </a:glow>
-                      </a:effectLst>
                       <a:latin typeface="+mn-lt"/>
                       <a:ea typeface="+mn-ea"/>
                       <a:cs typeface="+mn-cs"/>
@@ -4635,7 +4366,7 @@
                   <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
-              <c:dLblPos val="bestFit"/>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="1"/>
@@ -4666,13 +4397,8 @@
                 <a:pPr>
                   <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="bg1"/>
+                      <a:schemeClr val="accent3"/>
                     </a:solidFill>
-                    <a:effectLst>
-                      <a:glow rad="76200">
-                        <a:schemeClr val="tx1"/>
-                      </a:glow>
-                    </a:effectLst>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
@@ -4681,7 +4407,7 @@
                 <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:txPr>
-            <c:dLblPos val="bestFit"/>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="1"/>
@@ -4716,10 +4442,10 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>684912.47272727266</c:v>
+                  <c:v>127816.54944242424</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>201786.07120000003</c:v>
+                  <c:v>202404.21090000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4952,17 +4678,9 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                      <a:ln w="12700" cap="flat">
-                        <a:noFill/>
-                      </a:ln>
                       <a:solidFill>
-                        <a:schemeClr val="bg1"/>
+                        <a:schemeClr val="accent5"/>
                       </a:solidFill>
-                      <a:effectLst>
-                        <a:glow rad="76200">
-                          <a:schemeClr val="tx1"/>
-                        </a:glow>
-                      </a:effectLst>
                       <a:latin typeface="+mn-lt"/>
                       <a:ea typeface="+mn-ea"/>
                       <a:cs typeface="+mn-cs"/>
@@ -4971,7 +4689,7 @@
                   <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
-              <c:dLblPos val="bestFit"/>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="1"/>
@@ -5001,17 +4719,12 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                      <a:ln w="12700" cap="flat">
+                      <a:ln w="0">
                         <a:noFill/>
                       </a:ln>
                       <a:solidFill>
-                        <a:schemeClr val="bg1"/>
+                        <a:schemeClr val="accent4"/>
                       </a:solidFill>
-                      <a:effectLst>
-                        <a:glow rad="76200">
-                          <a:schemeClr val="tx1"/>
-                        </a:glow>
-                      </a:effectLst>
                       <a:latin typeface="+mn-lt"/>
                       <a:ea typeface="+mn-ea"/>
                       <a:cs typeface="+mn-cs"/>
@@ -5020,7 +4733,7 @@
                   <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
-              <c:dLblPos val="bestFit"/>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="1"/>
@@ -5050,17 +4763,9 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                      <a:ln w="12700" cap="flat">
-                        <a:noFill/>
-                      </a:ln>
                       <a:solidFill>
-                        <a:schemeClr val="bg1"/>
+                        <a:schemeClr val="accent6"/>
                       </a:solidFill>
-                      <a:effectLst>
-                        <a:glow rad="76200">
-                          <a:schemeClr val="tx1"/>
-                        </a:glow>
-                      </a:effectLst>
                       <a:latin typeface="+mn-lt"/>
                       <a:ea typeface="+mn-ea"/>
                       <a:cs typeface="+mn-cs"/>
@@ -5069,7 +4774,7 @@
                   <a:endParaRPr lang="en-US"/>
                 </a:p>
               </c:txPr>
-              <c:dLblPos val="bestFit"/>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="1"/>
@@ -5097,17 +4802,9 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-                    <a:ln w="12700" cap="flat">
-                      <a:noFill/>
-                    </a:ln>
                     <a:solidFill>
-                      <a:schemeClr val="bg1"/>
+                      <a:srgbClr val="DFC27D"/>
                     </a:solidFill>
-                    <a:effectLst>
-                      <a:glow rad="76200">
-                        <a:schemeClr val="tx1"/>
-                      </a:glow>
-                    </a:effectLst>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
                     <a:cs typeface="+mn-cs"/>
@@ -5116,7 +4813,7 @@
                 <a:endParaRPr lang="en-US"/>
               </a:p>
             </c:txPr>
-            <c:dLblPos val="bestFit"/>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="1"/>
@@ -5152,13 +4849,13 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>4472064.93</c:v>
+                  <c:v>1454221.3599999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>223589.91</c:v>
+                  <c:v>148361.25999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>661623.19000000006</c:v>
+                  <c:v>675217.69000000006</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5333,40 +5030,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>Oct 23</c:v>
+                  <c:v>Jan 24</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Nov 23</c:v>
+                  <c:v>Feb 24</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Dec 23</c:v>
+                  <c:v>Mar 24</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Jan 24</c:v>
+                  <c:v>Apr 24</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Feb 24</c:v>
+                  <c:v>May 24</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Mar 24</c:v>
+                  <c:v>Jun 24</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Apr 24</c:v>
+                  <c:v>Jul 24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>May 24</c:v>
+                  <c:v>Aug 24</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Jun 24</c:v>
+                  <c:v>Sep 24</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Jul 24</c:v>
+                  <c:v>Oct 24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Aug 24</c:v>
+                  <c:v>Nov 24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sep 24</c:v>
+                  <c:v>Dec 24</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5378,40 +5075,40 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>336267.31</c:v>
+                  <c:v>106397.86</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>337009.91999999998</c:v>
+                  <c:v>95101.49</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>403169.72</c:v>
+                  <c:v>100800.73</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>431726.45</c:v>
+                  <c:v>121946.65</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>361043.48</c:v>
+                  <c:v>117553.12999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>383119.25</c:v>
+                  <c:v>137534.25</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>394258.4</c:v>
+                  <c:v>151332.35</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>340182.89</c:v>
+                  <c:v>141123.71</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>359558.26</c:v>
+                  <c:v>131091.88999999998</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>397363.86</c:v>
+                  <c:v>119489.42</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>376165.72</c:v>
+                  <c:v>115818.54000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>352199.67</c:v>
+                  <c:v>116031.34</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5465,40 +5162,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>Oct 23</c:v>
+                  <c:v>Jan 24</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Nov 23</c:v>
+                  <c:v>Feb 24</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Dec 23</c:v>
+                  <c:v>Mar 24</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Jan 24</c:v>
+                  <c:v>Apr 24</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Feb 24</c:v>
+                  <c:v>May 24</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Mar 24</c:v>
+                  <c:v>Jun 24</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Apr 24</c:v>
+                  <c:v>Jul 24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>May 24</c:v>
+                  <c:v>Aug 24</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Jun 24</c:v>
+                  <c:v>Sep 24</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Jul 24</c:v>
+                  <c:v>Oct 24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Aug 24</c:v>
+                  <c:v>Nov 24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sep 24</c:v>
+                  <c:v>Dec 24</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5510,40 +5207,40 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>17843.61</c:v>
+                  <c:v>3727.2400000000002</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>17843.61</c:v>
+                  <c:v>3654.9300000000003</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>20304.8</c:v>
+                  <c:v>4105.5200000000004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>21535.39</c:v>
+                  <c:v>4318.84</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>17228.310000000001</c:v>
+                  <c:v>4585.8</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>18458.91</c:v>
+                  <c:v>26620.42</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>19689.5</c:v>
+                  <c:v>29423.26</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>17843.61</c:v>
+                  <c:v>29498.550000000003</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>18271.48</c:v>
+                  <c:v>26660.23</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>19189.689999999999</c:v>
+                  <c:v>4596.1099999999997</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>17390.66</c:v>
+                  <c:v>6038.83</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>17990.34</c:v>
+                  <c:v>5131.53</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5597,40 +5294,40 @@
               <c:strCache>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>Oct 23</c:v>
+                  <c:v>Jan 24</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Nov 23</c:v>
+                  <c:v>Feb 24</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>Dec 23</c:v>
+                  <c:v>Mar 24</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>Jan 24</c:v>
+                  <c:v>Apr 24</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>Feb 24</c:v>
+                  <c:v>May 24</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>Mar 24</c:v>
+                  <c:v>Jun 24</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Apr 24</c:v>
+                  <c:v>Jul 24</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>May 24</c:v>
+                  <c:v>Aug 24</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Jun 24</c:v>
+                  <c:v>Sep 24</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>Jul 24</c:v>
+                  <c:v>Oct 24</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>Aug 24</c:v>
+                  <c:v>Nov 24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>Sep 24</c:v>
+                  <c:v>Dec 24</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -5642,40 +5339,40 @@
                 <c:formatCode>#,##0_);\(#,##0\)</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>49724.82</c:v>
+                  <c:v>87857.74</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13191.5</c:v>
+                  <c:v>65523.329999999994</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>43547.51</c:v>
+                  <c:v>66562.8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>251777.42</c:v>
+                  <c:v>52165.7</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>58848.990000000005</c:v>
+                  <c:v>49743.42</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-3183.3199999999997</c:v>
+                  <c:v>46165.399999999994</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>61041.850000000006</c:v>
+                  <c:v>48984.39</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>42994.85</c:v>
+                  <c:v>50635.75</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>37352.270000000004</c:v>
+                  <c:v>51575.020000000004</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>35079.659999999996</c:v>
+                  <c:v>53352.630000000005</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>34223.160000000003</c:v>
+                  <c:v>75418.23</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>37024.480000000003</c:v>
+                  <c:v>27233.280000000002</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10402,6 +10099,12 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Alex Rios" id="{5B3192E5-3795-49D5-84DE-4B50D72ACC51}" userId="2f3315927d3711d0" providerId="Windows Live"/>
+</personList>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -10598,18 +10301,29 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C7" dT="2025-03-27T21:00:04.83" personId="{5B3192E5-3795-49D5-84DE-4B50D72ACC51}" id="{83BABB99-64A9-4C76-931E-7394AAFD09FD}">
+    <text>Values being added from account numbers in order:  (501-00) + (501-06) + (502-09)</text>
+  </threadedComment>
+  <threadedComment ref="L7" dT="2025-03-27T20:18:04.27" personId="{5B3192E5-3795-49D5-84DE-4B50D72ACC51}" id="{D1BC6906-84CA-4A7C-902B-5F76AE15F688}">
+    <text>Values being added from account numbers in order:  (501-00) + (948-03) + (460-18) + (50-303) + (3-4959) + (17427) + (3-4958) + (42923) + (3-4898)</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:W985"/>
-  <sheetFormatPr defaultColWidth="12.73046875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="23" width="15.86328125" customWidth="1"/>
+    <col min="1" max="23" width="15.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="99.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:23" ht="100.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A1" s="3"/>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -10625,26 +10339,26 @@
       <c r="M1" s="25"/>
       <c r="N1" s="25"/>
     </row>
-    <row r="2" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="3"/>
-      <c r="B2" s="122" t="s">
+      <c r="B2" s="103" t="s">
         <v>33</v>
       </c>
-      <c r="C2" s="123"/>
-      <c r="D2" s="123"/>
-      <c r="E2" s="123"/>
-      <c r="F2" s="123"/>
-      <c r="G2" s="123"/>
-      <c r="H2" s="123"/>
-      <c r="I2" s="124"/>
+      <c r="C2" s="104"/>
+      <c r="D2" s="104"/>
+      <c r="E2" s="104"/>
+      <c r="F2" s="104"/>
+      <c r="G2" s="104"/>
+      <c r="H2" s="104"/>
+      <c r="I2" s="105"/>
       <c r="J2" s="3"/>
-      <c r="K2" s="116" t="str">
+      <c r="K2" s="97" t="str">
         <f>_xlfn.CONCAT(Q2," Usage and Cost by Month")</f>
         <v>Natural Gas Usage and Cost by Month</v>
       </c>
-      <c r="L2" s="117"/>
-      <c r="M2" s="117"/>
-      <c r="N2" s="118"/>
+      <c r="L2" s="98"/>
+      <c r="M2" s="98"/>
+      <c r="N2" s="99"/>
       <c r="P2" s="71" t="s">
         <v>48</v>
       </c>
@@ -10652,29 +10366,29 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:23" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:23" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A3" s="3"/>
-      <c r="B3" s="125"/>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="127"/>
+      <c r="B3" s="106"/>
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
+      <c r="E3" s="107"/>
+      <c r="F3" s="107"/>
+      <c r="G3" s="107"/>
+      <c r="H3" s="107"/>
+      <c r="I3" s="108"/>
       <c r="J3" s="4"/>
-      <c r="K3" s="119"/>
-      <c r="L3" s="120"/>
-      <c r="M3" s="120"/>
-      <c r="N3" s="121"/>
+      <c r="K3" s="100"/>
+      <c r="L3" s="101"/>
+      <c r="M3" s="101"/>
+      <c r="N3" s="102"/>
       <c r="P3" s="71" t="s">
         <v>49</v>
       </c>
       <c r="Q3" s="79" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="3"/>
       <c r="B4" s="34" t="s">
         <v>0</v>
@@ -10722,10 +10436,10 @@
       </c>
       <c r="Q4" s="75">
         <f>VLOOKUP(Q2,P7:W14,MATCH(Q3,P6:W6,0),FALSE)</f>
-        <v>1.036</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="3"/>
       <c r="B5" s="5" t="s">
         <v>14</v>
@@ -10768,10 +10482,10 @@
         <v>50</v>
       </c>
       <c r="Q5" s="80">
-        <v>45200</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+        <v>45293</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A6" s="3"/>
       <c r="B6" s="37" t="s">
         <v>15</v>
@@ -10803,7 +10517,7 @@
       </c>
       <c r="L6" s="38" t="str">
         <f>_xlfn.CONCAT("[",Q3,"]")</f>
-        <v>[Mcf]</v>
+        <v>[Therm]</v>
       </c>
       <c r="M6" s="38" t="s">
         <v>11</v>
@@ -10836,50 +10550,56 @@
         <v>44</v>
       </c>
     </row>
-    <row r="7" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="3"/>
       <c r="B7" s="23" t="str">
         <f>TEXT(EDATE($Q$5,0),"mmm yy")</f>
-        <v>Oct 23</v>
+        <v>Jan 24</v>
       </c>
       <c r="C7" s="81">
-        <v>4981000</v>
+        <f>49445 + 24298 + 850145 + 933</f>
+        <v>924821</v>
       </c>
       <c r="D7" s="81">
-        <v>336267.31</v>
+        <f>5674.09 + 2788.29 + 97854.34 + 81.14</f>
+        <v>106397.86</v>
       </c>
       <c r="E7" s="81">
-        <v>11081</v>
+        <f>97.7 + 163.5 + 1250.7</f>
+        <v>1511.9</v>
       </c>
       <c r="F7" s="81">
-        <v>17843.61</v>
+        <f>484.55 + 810.89 + 2431.8</f>
+        <v>3727.2400000000002</v>
       </c>
       <c r="G7" s="81">
-        <f>470137.29-D7-F7</f>
-        <v>116026.36999999998</v>
+        <f>H7-D7-F7</f>
+        <v>1308.3700000000003</v>
       </c>
       <c r="H7" s="81">
-        <f t="shared" ref="H7:H8" si="0">G7+D7+F7</f>
-        <v>470137.29</v>
+        <f>6529.45 + 3969.99 + 100656.95 + 277.08</f>
+        <v>111433.47</v>
       </c>
       <c r="I7" s="84">
         <f>C7*0.003412/0.33</f>
-        <v>51500.521212121217</v>
+        <v>9562.0886424242435</v>
       </c>
       <c r="J7" s="4"/>
       <c r="K7" s="23" t="str">
-        <f t="shared" ref="K7:K18" si="1">B7</f>
-        <v>Oct 23</v>
+        <f t="shared" ref="K7:K18" si="0">B7</f>
+        <v>Jan 24</v>
       </c>
       <c r="L7" s="87">
-        <v>11617.8</v>
+        <f>1661.844 + 1463.878 + 3506.762 + 78427.317 + (7910 * 3) + 84780</f>
+        <v>193569.80099999998</v>
       </c>
       <c r="M7" s="8">
         <f>L7*$Q$4</f>
-        <v>12036.040799999999</v>
+        <v>19356.980099999997</v>
       </c>
       <c r="N7" s="90">
-        <v>49724.82</v>
+        <f>687.61 + 663.69 + 1205.46 + 21490.25 + 827.07 + 1981.19 + 938.86 + 60063.61</f>
+        <v>87857.74</v>
       </c>
       <c r="P7" s="68" t="s">
         <v>29</v>
@@ -10900,50 +10620,56 @@
       <c r="V7" s="76"/>
       <c r="W7" s="76"/>
     </row>
-    <row r="8" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="3"/>
       <c r="B8" s="24" t="str">
         <f>TEXT(EDATE($Q$5,1),"mmm yy")</f>
-        <v>Nov 23</v>
+        <v>Feb 24</v>
       </c>
       <c r="C8" s="82">
-        <v>4992000</v>
+        <f>51115 + 20456 + 752185 + 797</f>
+        <v>824553</v>
       </c>
       <c r="D8" s="82">
-        <v>337009.91999999998</v>
+        <f>5887.74 + 2355.45 + 86788.98 + 69.32</f>
+        <v>95101.49</v>
       </c>
       <c r="E8" s="82">
-        <v>10200</v>
+        <f>95.8 + 156.3 + 1335.6</f>
+        <v>1587.6999999999998</v>
       </c>
       <c r="F8" s="82">
-        <v>17843.61</v>
+        <f>475.13 + 775.19 + 2404.61</f>
+        <v>3654.9300000000003</v>
       </c>
       <c r="G8" s="82">
-        <f>470813.2-D8-F8</f>
-        <v>115959.67000000003</v>
+        <f t="shared" ref="G8:G18" si="1">H8-D8-F8</f>
+        <v>1308.3699999999881</v>
       </c>
       <c r="H8" s="82">
-        <f t="shared" si="0"/>
-        <v>470813.2</v>
+        <f>6733.68 + 3501.45 + 89564.4 +265.26</f>
+        <v>100064.79</v>
       </c>
       <c r="I8" s="85">
         <f>C8*0.003412/0.33</f>
-        <v>51614.254545454547</v>
+        <v>8525.3782909090896</v>
       </c>
       <c r="J8" s="4"/>
       <c r="K8" s="24" t="str">
-        <f t="shared" si="1"/>
-        <v>Nov 23</v>
+        <f t="shared" si="0"/>
+        <v>Feb 24</v>
       </c>
       <c r="L8" s="88">
-        <v>24415.3</v>
+        <f>1393.253 + 1368.641 + 3480.577 + 73995.434 + (7160 * 3) + 73994.434</f>
+        <v>175712.33899999998</v>
       </c>
       <c r="M8" s="10">
         <f>L8*$Q$4</f>
-        <v>25294.250800000002</v>
+        <v>17571.233899999999</v>
       </c>
       <c r="N8" s="91">
-        <v>13191.5</v>
+        <f>640.25 + 646.63+ 1197.85 + 21122.78 + 802.13 + 2040 + 816.55 + 37458.29 + 798.85</f>
+        <v>65523.329999999994</v>
       </c>
       <c r="P8" s="67" t="s">
         <v>31</v>
@@ -10962,50 +10688,56 @@
       <c r="V8" s="76"/>
       <c r="W8" s="76"/>
     </row>
-    <row r="9" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="3"/>
       <c r="B9" s="24" t="str">
         <f>TEXT(EDATE($Q$5,2),"mmm yy")</f>
-        <v>Dec 23</v>
+        <v>Mar 24</v>
       </c>
       <c r="C9" s="82">
-        <v>5972000</v>
+        <f>48426 + 22418 + 794725 + 696</f>
+        <v>866265</v>
       </c>
       <c r="D9" s="82">
-        <v>403169.72</v>
+        <f>5637.5 + 2611.28 + 92485.89 + 66.06</f>
+        <v>100800.73</v>
       </c>
       <c r="E9" s="82">
-        <v>10744</v>
+        <f>98.6 + 178.5 + 1517</f>
+        <v>1794.1</v>
       </c>
       <c r="F9" s="82">
-        <v>20304.8</v>
+        <f>489.02 + 885.29 + 2731.21</f>
+        <v>4105.5200000000004</v>
       </c>
       <c r="G9" s="82">
-        <f>556736.92-D9-F9</f>
-        <v>133262.40000000008</v>
+        <f t="shared" si="1"/>
+        <v>1308.369999999999</v>
       </c>
       <c r="H9" s="82">
-        <f>G9+D9+F9</f>
-        <v>556736.92000000016</v>
+        <f>6497.33 + 3867.38 + 95587.91 + 262</f>
+        <v>106214.62</v>
       </c>
       <c r="I9" s="85">
         <f t="shared" ref="I9:I17" si="2">C9*0.003412/0.33</f>
-        <v>61746.860606060603</v>
+        <v>8956.6550909090911</v>
       </c>
       <c r="J9" s="4"/>
       <c r="K9" s="24" t="str">
-        <f t="shared" si="1"/>
-        <v>Dec 23</v>
+        <f t="shared" si="0"/>
+        <v>Mar 24</v>
       </c>
       <c r="L9" s="88">
-        <v>27255.5</v>
+        <f>664.524 + 1445.687 + 2961.056 + 80360.044 + (5980 * 3) + 80360.044</f>
+        <v>183731.35499999998</v>
       </c>
       <c r="M9" s="10">
         <f t="shared" ref="M9:M17" si="3">L9*$Q$4</f>
-        <v>28236.698</v>
+        <v>18373.1355</v>
       </c>
       <c r="N9" s="91">
-        <v>43547.51</v>
+        <f>517.35 + 668.77 + 1098.76 + 20625.4 + 847.34 + 1735.52 +389.44 + 40680.22</f>
+        <v>66562.8</v>
       </c>
       <c r="P9" s="69" t="s">
         <v>47</v>
@@ -11024,50 +10756,56 @@
       <c r="V9" s="77"/>
       <c r="W9" s="76"/>
     </row>
-    <row r="10" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="3"/>
       <c r="B10" s="24" t="str">
         <f>TEXT(EDATE($Q$5,3),"mmm yy")</f>
-        <v>Jan 24</v>
+        <v>Apr 24</v>
       </c>
       <c r="C10" s="82">
-        <v>6395000</v>
+        <f>53136 + 24812 + 964606 + 685</f>
+        <v>1043239</v>
       </c>
       <c r="D10" s="82">
-        <v>431726.45</v>
+        <f>6218.15 + 2905.02 + 112753.54 + 69.94</f>
+        <v>121946.65</v>
       </c>
       <c r="E10" s="82">
-        <v>10744</v>
+        <f>108.4 + 187.9 + 1582.6</f>
+        <v>1878.8999999999999</v>
       </c>
       <c r="F10" s="82">
-        <v>21535.39</v>
+        <f>537.62 + 931.91 + 2849.31</f>
+        <v>4318.84</v>
       </c>
       <c r="G10" s="82">
-        <f>588492.71-D10-F10</f>
-        <v>135230.86999999994</v>
+        <f t="shared" si="1"/>
+        <v>1308.3700000000208</v>
       </c>
       <c r="H10" s="82">
-        <f t="shared" ref="H10:H18" si="4">G10+D10+F10</f>
-        <v>588492.71</v>
+        <f>7126.58 +4207.74 + 115973.66 + 265.88</f>
+        <v>127573.86000000002</v>
       </c>
       <c r="I10" s="85">
         <f t="shared" si="2"/>
-        <v>66120.42424242424</v>
+        <v>10786.458993939394</v>
       </c>
       <c r="J10" s="4"/>
       <c r="K10" s="24" t="str">
-        <f t="shared" si="1"/>
-        <v>Jan 24</v>
+        <f t="shared" si="0"/>
+        <v>Apr 24</v>
       </c>
       <c r="L10" s="88">
-        <v>36376.800000000003</v>
+        <f>892.452 + 1335.8 + 2590.27 + 77078.944 + (4920 * 3) + 77078.944</f>
+        <v>173736.41</v>
       </c>
       <c r="M10" s="10">
         <f t="shared" si="3"/>
-        <v>37686.364800000003</v>
+        <v>17373.641</v>
       </c>
       <c r="N10" s="91">
-        <v>251777.42</v>
+        <f>308.23 + 424.41 + 504.3 + 9073.63 + 794.67 + 1518.17 + 523.04 + 39019.25</f>
+        <v>52165.7</v>
       </c>
       <c r="P10" s="69" t="s">
         <v>34</v>
@@ -11082,50 +10820,56 @@
       <c r="V10" s="76"/>
       <c r="W10" s="76"/>
     </row>
-    <row r="11" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="3"/>
       <c r="B11" s="24" t="str">
         <f>TEXT(EDATE($Q$5,4),"mmm yy")</f>
-        <v>Feb 24</v>
+        <v>May 24</v>
       </c>
       <c r="C11" s="82">
-        <v>5348000</v>
+        <f>54461 + 27050 + 922383 + 548</f>
+        <v>1004442</v>
       </c>
       <c r="D11" s="82">
-        <v>361043.48</v>
+        <f>6376.35 + 3166.56 + 107953.18 + 57.04</f>
+        <v>117553.12999999999</v>
       </c>
       <c r="E11" s="82">
-        <v>11184</v>
+        <f>117.2 + 209.8 + 1633</f>
+        <v>1960</v>
       </c>
       <c r="F11" s="82">
-        <v>17228.310000000001</v>
+        <f>583.38 + 1044.15 + 2958.27</f>
+        <v>4585.8</v>
       </c>
       <c r="G11" s="82">
-        <f>479137.96-D11-F11</f>
-        <v>100866.17000000004</v>
+        <f t="shared" si="1"/>
+        <v>2950.5600000000004</v>
       </c>
       <c r="H11" s="82">
-        <f>G11+D11+F11</f>
-        <v>479137.96</v>
+        <f>7330.54 + 4581.52 + 112924.45 + 252.98</f>
+        <v>125089.48999999999</v>
       </c>
       <c r="I11" s="85">
         <f t="shared" si="2"/>
-        <v>55295.078787878789</v>
+        <v>10385.321527272727</v>
       </c>
       <c r="J11" s="4"/>
       <c r="K11" s="24" t="str">
-        <f t="shared" si="1"/>
-        <v>Feb 24</v>
+        <f t="shared" si="0"/>
+        <v>May 24</v>
       </c>
       <c r="L11" s="88">
-        <v>29873.599999999999</v>
+        <f>343.83 + 335.261 + 2230.015 + 75278.224 + (3120 * 3) + 75278.224</f>
+        <v>162825.554</v>
       </c>
       <c r="M11" s="10">
         <f t="shared" si="3"/>
-        <v>30949.049599999998</v>
+        <v>16282.555400000001</v>
       </c>
       <c r="N11" s="91">
-        <v>58848.990000000005</v>
+        <f>211.8 + 236.8 + 445.44 + 8496.06 + 207.07 + 1307.02 + 731.55 + 38107.68</f>
+        <v>49743.42</v>
       </c>
       <c r="P11" s="68" t="s">
         <v>32</v>
@@ -11140,50 +10884,56 @@
       <c r="V11" s="76"/>
       <c r="W11" s="78"/>
     </row>
-    <row r="12" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="3"/>
       <c r="B12" s="24" t="str">
         <f>TEXT(EDATE($Q$5,5),"mmm yy")</f>
-        <v>Mar 24</v>
+        <v>Jun 24</v>
       </c>
       <c r="C12" s="82">
-        <v>5675000</v>
+        <f>68384 + 39725 + 1067243 + 542</f>
+        <v>1175894</v>
       </c>
       <c r="D12" s="82">
-        <v>383119.25</v>
+        <f>7998.29 + 4640.86 + 124840.04 + 55.06</f>
+        <v>137534.25</v>
       </c>
       <c r="E12" s="82">
-        <v>11042</v>
+        <f>115.2 +203.7 +1920.2</f>
+        <v>2239.1</v>
       </c>
       <c r="F12" s="82">
-        <v>18458.91</v>
+        <f>1641.4 + 2902.16 + 22076.86</f>
+        <v>26620.42</v>
       </c>
       <c r="G12" s="82">
-        <f>511186.96-D12-F12</f>
-        <v>109608.80000000002</v>
+        <f t="shared" si="1"/>
+        <v>1308.3699999999808</v>
       </c>
       <c r="H12" s="82">
-        <f t="shared" si="4"/>
-        <v>511186.96</v>
+        <f>10010.5 + 7913.83 + 147287.71 + 251</f>
+        <v>165463.03999999998</v>
       </c>
       <c r="I12" s="85">
         <f t="shared" si="2"/>
-        <v>58676.060606060608</v>
+        <v>12158.031296969697</v>
       </c>
       <c r="J12" s="4"/>
       <c r="K12" s="24" t="str">
-        <f t="shared" si="1"/>
-        <v>Mar 24</v>
+        <f t="shared" si="0"/>
+        <v>Jun 24</v>
       </c>
       <c r="L12" s="88">
-        <v>25421.8</v>
+        <f>323.166 + 13.911 + 1958.675 + 72164.119 + (1640 * 3) + 72164.119</f>
+        <v>151543.99</v>
       </c>
       <c r="M12" s="10">
         <f t="shared" si="3"/>
-        <v>26336.984799999998</v>
+        <v>15154.398999999999</v>
       </c>
       <c r="N12" s="91">
-        <v>-3183.3199999999997</v>
+        <f>206.82 + 180.83 + 361.74 + 7539.26 + 8.16 + 1147.97 + 189.38 + 36531.24</f>
+        <v>46165.399999999994</v>
       </c>
       <c r="P12" s="68" t="s">
         <v>35</v>
@@ -11198,50 +10948,56 @@
       <c r="V12" s="76"/>
       <c r="W12" s="78"/>
     </row>
-    <row r="13" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="3"/>
       <c r="B13" s="24" t="str">
         <f>TEXT(EDATE($Q$5,6),"mmm yy")</f>
-        <v>Apr 24</v>
+        <v>Jul 24</v>
       </c>
       <c r="C13" s="82">
-        <v>5840000</v>
+        <f>65104 + 51706 + 1166005 + 543</f>
+        <v>1283358</v>
       </c>
       <c r="D13" s="82">
-        <v>394258.4</v>
+        <f>7686.65 + 6089.2 + 137501.4 + 55.1</f>
+        <v>151332.35</v>
       </c>
       <c r="E13" s="82">
-        <v>11042</v>
+        <f>120.4 + 247.5 + 2026.1</f>
+        <v>2394</v>
       </c>
       <c r="F13" s="82">
-        <v>19689.5</v>
+        <f>1716.36 + 3528.24 +24178.66</f>
+        <v>29423.26</v>
       </c>
       <c r="G13" s="82">
-        <f>530210.33-D13-F13</f>
-        <v>116262.42999999993</v>
+        <f t="shared" si="1"/>
+        <v>1308.3700000000063</v>
       </c>
       <c r="H13" s="82">
-        <f t="shared" si="4"/>
-        <v>530210.32999999996</v>
+        <f>9773.82 + 9988.25 + 162050.87 + 251.04</f>
+        <v>182063.98</v>
       </c>
       <c r="I13" s="85">
         <f t="shared" si="2"/>
-        <v>60382.060606060608</v>
+        <v>13269.143927272728</v>
       </c>
       <c r="J13" s="4"/>
       <c r="K13" s="24" t="str">
-        <f t="shared" si="1"/>
-        <v>Apr 24</v>
+        <f t="shared" si="0"/>
+        <v>Jul 24</v>
       </c>
       <c r="L13" s="88">
-        <v>17141.900000000001</v>
+        <f>246.712 + 6.408 + 1889.031 + 76206.127 + (240 * 3) + 76206.127</f>
+        <v>155274.40499999997</v>
       </c>
       <c r="M13" s="10">
         <f t="shared" si="3"/>
-        <v>17759.008400000002</v>
+        <v>15527.440499999997</v>
       </c>
       <c r="N13" s="91">
-        <v>61041.850000000006</v>
+        <f>201.62 + 180.23 + 363.98 + 8405.55 + 3.79 + 1107.19 + 144.63 + 38577.4</f>
+        <v>48984.39</v>
       </c>
       <c r="P13" s="68" t="s">
         <v>36</v>
@@ -11256,50 +11012,56 @@
       <c r="V13" s="76"/>
       <c r="W13" s="78"/>
     </row>
-    <row r="14" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="3"/>
       <c r="B14" s="24" t="str">
         <f>TEXT(EDATE($Q$5,7),"mmm yy")</f>
-        <v>May 24</v>
+        <v>Aug 24</v>
       </c>
       <c r="C14" s="82">
-        <v>5039000</v>
+        <f>60014 + 49317 + 1079645 + 553</f>
+        <v>1189529</v>
       </c>
       <c r="D14" s="82">
-        <v>340182.89</v>
+        <f>7131.07 + 5831.39 + 128105.06 + 56.19</f>
+        <v>141123.71</v>
       </c>
       <c r="E14" s="82">
-        <v>10588</v>
+        <f>119.3 + 211 + 2081.5</f>
+        <v>2411.8000000000002</v>
       </c>
       <c r="F14" s="82">
-        <v>17843.61</v>
+        <f>1709.7 + 2949.06 + 24839.79</f>
+        <v>29498.550000000003</v>
       </c>
       <c r="G14" s="82">
-        <f>462102.23-D14-F14</f>
-        <v>104075.72999999997</v>
+        <f t="shared" si="1"/>
+        <v>1308.8000000000029</v>
       </c>
       <c r="H14" s="82">
-        <f t="shared" si="4"/>
-        <v>462102.23</v>
+        <f>9211.58 + 9151.36 + 153315.99 + 252.13</f>
+        <v>171931.06</v>
       </c>
       <c r="I14" s="85">
         <f t="shared" si="2"/>
-        <v>52100.206060606055</v>
+        <v>12299.008933333333</v>
       </c>
       <c r="J14" s="4"/>
       <c r="K14" s="24" t="str">
-        <f t="shared" si="1"/>
-        <v>May 24</v>
+        <f t="shared" si="0"/>
+        <v>Aug 24</v>
       </c>
       <c r="L14" s="88">
-        <v>7114.5</v>
+        <f>277.685 + 3.204 + 1888.766 + 78821.863 + (2780 * 3) + 78821.863</f>
+        <v>168153.38099999999</v>
       </c>
       <c r="M14" s="10">
         <f t="shared" si="3"/>
-        <v>7370.6220000000003</v>
-      </c>
-      <c r="N14" s="109">
-        <v>42994.85</v>
+        <v>16815.338100000001</v>
+      </c>
+      <c r="N14" s="91">
+        <f>204.65 + 179.95 + 365.82 + 8688.52 + 1.95 + 984.04 + 309.27 + 39901.55</f>
+        <v>50635.75</v>
       </c>
       <c r="P14" s="68" t="s">
         <v>37</v>
@@ -11316,241 +11078,265 @@
         <v>83.34</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="3"/>
       <c r="B15" s="24" t="str">
         <f>TEXT(EDATE($Q$5,8),"mmm yy")</f>
-        <v>Jun 24</v>
+        <v>Sep 24</v>
       </c>
       <c r="C15" s="82">
-        <v>5326000</v>
+        <f>59763 + 46208 + 997169 + 642</f>
+        <v>1103782</v>
       </c>
       <c r="D15" s="82">
-        <v>359558.26</v>
+        <f>7110.15 + 5470.45 + 118449.8 + 61.49</f>
+        <v>131091.88999999998</v>
       </c>
       <c r="E15" s="82">
-        <v>11094</v>
+        <f>102.2 + 254.6 + 1864.8</f>
+        <v>2221.6</v>
       </c>
       <c r="F15" s="82">
-        <v>18271.48</v>
+        <f>1466.65 + 3653.71 +21539.87</f>
+        <v>26660.23</v>
       </c>
       <c r="G15" s="82">
-        <f>485210.72-D15-F15</f>
-        <v>107380.97999999997</v>
+        <f t="shared" si="1"/>
+        <v>1308.2600000000202</v>
       </c>
       <c r="H15" s="82">
-        <f t="shared" si="4"/>
-        <v>485210.72</v>
+        <f>8947.5 + 9494.97 + 140360.48 +257.43</f>
+        <v>159060.38</v>
       </c>
       <c r="I15" s="85">
         <f t="shared" si="2"/>
-        <v>55067.612121212122</v>
+        <v>11412.436921212122</v>
       </c>
       <c r="J15" s="4"/>
       <c r="K15" s="24" t="str">
-        <f t="shared" si="1"/>
-        <v>Jun 24</v>
+        <f t="shared" si="0"/>
+        <v>Sep 24</v>
       </c>
       <c r="L15" s="88">
-        <v>4047</v>
+        <f>306.818 + 2.138 + 2021.796 + 80224.153 + (3810 * 3) + 80224.153</f>
+        <v>174209.05800000002</v>
       </c>
       <c r="M15" s="10">
         <f t="shared" si="3"/>
-        <v>4192.692</v>
+        <v>17420.905800000004</v>
       </c>
       <c r="N15" s="91">
-        <v>37352.270000000004</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+        <f>207.28 + 179.85 + 448.12 + 8840.22 + 1.26 + 1107.02 + 179.84 + 40611.43</f>
+        <v>51575.020000000004</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="3"/>
       <c r="B16" s="24" t="str">
         <f>TEXT(EDATE($Q$5,9),"mmm yy")</f>
-        <v>Jul 24</v>
+        <v>Oct 24</v>
       </c>
       <c r="C16" s="82">
-        <v>5886000</v>
+        <f>46443 + 46057 + 907624 + 747</f>
+        <v>1000871</v>
       </c>
       <c r="D16" s="82">
-        <v>397363.86</v>
+        <f>5555.4 + 5466.83 + 108393.69 + 73.5</f>
+        <v>119489.42</v>
       </c>
       <c r="E16" s="82">
-        <v>12299</v>
+        <f>91.8 + 147.9 + 1688.4</f>
+        <v>1928.1000000000001</v>
       </c>
       <c r="F16" s="82">
-        <v>19189.689999999999</v>
+        <f>469.36 + 755.76 + 3370.99</f>
+        <v>4596.1099999999997</v>
       </c>
       <c r="G16" s="82">
-        <f>531357.16-D16-F16</f>
-        <v>114803.61000000004</v>
+        <f t="shared" si="1"/>
+        <v>1312.5100000000102</v>
       </c>
       <c r="H16" s="82">
-        <f t="shared" si="4"/>
-        <v>531357.16</v>
+        <f>6395.57 + 6593.4 + 112135.49 + 273.58</f>
+        <v>125398.04000000001</v>
       </c>
       <c r="I16" s="85">
         <f t="shared" si="2"/>
-        <v>60857.672727272722</v>
+        <v>10348.399551515151</v>
       </c>
       <c r="J16" s="4"/>
       <c r="K16" s="24" t="str">
-        <f t="shared" si="1"/>
-        <v>Jul 24</v>
+        <f t="shared" si="0"/>
+        <v>Oct 24</v>
       </c>
       <c r="L16" s="88">
-        <v>2940.7</v>
+        <f>317.202 + 2.136 +2569.583 + 81530.144 + (5380 * 3) + 81530.144</f>
+        <v>182089.209</v>
       </c>
       <c r="M16" s="10">
         <f t="shared" si="3"/>
-        <v>3046.5652</v>
+        <v>18208.920900000001</v>
       </c>
       <c r="N16" s="91">
-        <v>35079.659999999996</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+        <f>241.83 + 199.35 + 1233.41 + 9033.35 + 1.26 + 1184.96 + 185.93 + 41272.54</f>
+        <v>53352.630000000005</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="3"/>
       <c r="B17" s="24" t="str">
         <f>TEXT(EDATE($Q$5,10),"mmm yy")</f>
-        <v>Aug 24</v>
+        <v>Nov 24</v>
       </c>
       <c r="C17" s="82">
-        <v>5572000</v>
+        <f>40838 + 43428 + 887115 + 769</f>
+        <v>972150</v>
       </c>
       <c r="D17" s="82">
-        <v>376165.72</v>
+        <f>4871.16 + 5131.67 + 105737.74 + 77.97</f>
+        <v>115818.54000000001</v>
       </c>
       <c r="E17" s="82">
-        <v>12390</v>
+        <f>82.3 + 141.6 +1879.9</f>
+        <v>2103.8000000000002</v>
       </c>
       <c r="F17" s="82">
-        <v>17390.66</v>
+        <f>425.6 + 732.26 + 4880.97</f>
+        <v>6038.83</v>
       </c>
       <c r="G17" s="82">
-        <f>496860.92-D17-F17</f>
-        <v>103304.54000000001</v>
+        <f t="shared" si="1"/>
+        <v>1326.6899999999896</v>
       </c>
       <c r="H17" s="82">
-        <f t="shared" si="4"/>
-        <v>496860.92</v>
+        <f>5667.57 + 6234.74 + 110989.52 + 292.23</f>
+        <v>123184.06</v>
       </c>
       <c r="I17" s="85">
         <f t="shared" si="2"/>
-        <v>57611.103030303027</v>
+        <v>10051.441818181818</v>
       </c>
       <c r="J17" s="4"/>
       <c r="K17" s="24" t="str">
-        <f t="shared" si="1"/>
-        <v>Aug 24</v>
+        <f t="shared" si="0"/>
+        <v>Nov 24</v>
       </c>
       <c r="L17" s="88">
-        <v>3393.2</v>
+        <f>336.426 + 39.517 + 3688.764 + 92594.446 + (5290 * 3) + 92594.446</f>
+        <v>205123.59899999999</v>
       </c>
       <c r="M17" s="10">
         <f t="shared" si="3"/>
-        <v>3515.3552</v>
+        <v>20512.359899999999</v>
       </c>
       <c r="N17" s="91">
-        <v>34223.160000000003</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+        <f>579.8 + 509.1 + 1424.23 + 24305.14 + 23.15 + 1506.05 + 197.19 + 46873.57</f>
+        <v>75418.23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A18" s="3"/>
       <c r="B18" s="40" t="str">
         <f>TEXT(EDATE($Q$5,11),"mmm yy")</f>
-        <v>Sep 24</v>
+        <v>Dec 24</v>
       </c>
       <c r="C18" s="83">
-        <v>5217000</v>
+        <f>57266 + 41818 + 873231 + 874</f>
+        <v>973189</v>
       </c>
       <c r="D18" s="83">
-        <v>352199.67</v>
+        <f>6808.85 + 4947.75 + 104182.43 + 92.31</f>
+        <v>116031.34</v>
       </c>
       <c r="E18" s="83">
-        <v>11340</v>
+        <f>96.3 + 157.1 + 1471.7</f>
+        <v>1725.1</v>
       </c>
       <c r="F18" s="83">
-        <v>17990.34</v>
+        <f>498 + 812.41 + 3821.12</f>
+        <v>5131.53</v>
       </c>
       <c r="G18" s="83">
-        <f>475930.66-D18-F18</f>
-        <v>105740.65</v>
+        <f t="shared" si="1"/>
+        <v>1327.2200000000148</v>
       </c>
       <c r="H18" s="83">
-        <f t="shared" si="4"/>
-        <v>475930.66</v>
+        <f>7677.66 + 6131.5 + 108374.36 + 306.57</f>
+        <v>122490.09000000001</v>
       </c>
       <c r="I18" s="86">
         <f>C18*0.003412/0.33</f>
-        <v>53940.618181818187</v>
+        <v>10062.184448484848</v>
       </c>
       <c r="J18" s="4"/>
       <c r="K18" s="40" t="str">
-        <f t="shared" si="1"/>
-        <v>Sep 24</v>
+        <f t="shared" si="0"/>
+        <v>Dec 24</v>
       </c>
       <c r="L18" s="89">
-        <v>5176.1000000000004</v>
+        <f>1359.339 + 904.803 + 3506.762 + 75622.104 + (5560 * 3)</f>
+        <v>98073.008000000002</v>
       </c>
       <c r="M18" s="47">
         <f>L18*$Q$4</f>
-        <v>5362.4396000000006</v>
+        <v>9807.3008000000009</v>
       </c>
       <c r="N18" s="92">
-        <v>37024.480000000003</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+        <f>825.35 + 728.1 + 1205.46 + 20985.25 + 530.33 + 2162.06 + 796.73</f>
+        <v>27233.280000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A19" s="3"/>
       <c r="B19" s="41" t="s">
         <v>4</v>
       </c>
       <c r="C19" s="42">
-        <f t="shared" ref="C19:I19" si="5">SUM(C7:C18)</f>
-        <v>66243000</v>
+        <f t="shared" ref="C19:I19" si="4">SUM(C7:C18)</f>
+        <v>12362093</v>
       </c>
       <c r="D19" s="42">
-        <f t="shared" si="5"/>
-        <v>4472064.93</v>
+        <f t="shared" si="4"/>
+        <v>1454221.3599999999</v>
       </c>
       <c r="E19" s="42">
-        <f t="shared" si="5"/>
-        <v>133748</v>
+        <f t="shared" si="4"/>
+        <v>23756.099999999995</v>
       </c>
       <c r="F19" s="43">
-        <f t="shared" si="5"/>
-        <v>223589.91</v>
+        <f t="shared" si="4"/>
+        <v>148361.25999999998</v>
       </c>
       <c r="G19" s="43">
-        <f t="shared" si="5"/>
-        <v>1362522.22</v>
+        <f t="shared" si="4"/>
+        <v>17384.260000000031</v>
       </c>
       <c r="H19" s="42">
-        <f t="shared" si="5"/>
-        <v>6058177.0600000005</v>
+        <f t="shared" si="4"/>
+        <v>1619966.8800000001</v>
       </c>
       <c r="I19" s="44">
-        <f t="shared" si="5"/>
-        <v>684912.47272727266</v>
+        <f t="shared" si="4"/>
+        <v>127816.54944242424</v>
       </c>
       <c r="J19" s="4"/>
       <c r="K19" s="49" t="s">
         <v>17</v>
       </c>
       <c r="L19" s="50">
-        <f t="shared" ref="L19:N19" si="6">SUM(L7:L18)</f>
-        <v>194774.2</v>
+        <f t="shared" ref="L19:N19" si="5">SUM(L7:L18)</f>
+        <v>2024042.1089999997</v>
       </c>
       <c r="M19" s="50">
-        <f t="shared" si="6"/>
-        <v>201786.07120000003</v>
+        <f t="shared" si="5"/>
+        <v>202404.21090000001</v>
       </c>
       <c r="N19" s="51">
-        <f t="shared" si="6"/>
-        <v>661623.19000000006</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+        <f t="shared" si="5"/>
+        <v>675217.69000000006</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="3"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4"/>
@@ -11566,15 +11352,15 @@
       <c r="M20" s="14"/>
       <c r="N20" s="15"/>
     </row>
-    <row r="21" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:14" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="3"/>
-      <c r="B21" s="114" t="s">
+      <c r="B21" s="95" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="113"/>
+      <c r="C21" s="94"/>
       <c r="D21" s="16">
         <f>D19/C19</f>
-        <v>6.7510000000000001E-2</v>
+        <v>0.11763552984110376</v>
       </c>
       <c r="E21" s="17" t="s">
         <v>12</v>
@@ -11585,15 +11371,15 @@
       <c r="I21" s="3"/>
       <c r="J21" s="4"/>
     </row>
-    <row r="22" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:14" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="3"/>
-      <c r="B22" s="114" t="s">
+      <c r="B22" s="95" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="115"/>
+      <c r="C22" s="96"/>
       <c r="D22" s="18">
         <f>D19/I19</f>
-        <v>6.5293962485345842</v>
+        <v>11.377410564936765</v>
       </c>
       <c r="E22" s="19" t="s">
         <v>26</v>
@@ -11604,15 +11390,15 @@
       <c r="I22" s="30"/>
       <c r="J22" s="4"/>
     </row>
-    <row r="23" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:14" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="3"/>
-      <c r="B23" s="114" t="s">
+      <c r="B23" s="95" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="113"/>
+      <c r="C23" s="94"/>
       <c r="D23" s="20">
         <f>F19/E19</f>
-        <v>1.671725259443132</v>
+        <v>6.2451858680507328</v>
       </c>
       <c r="E23" s="17" t="s">
         <v>13</v>
@@ -11623,16 +11409,16 @@
       <c r="I23" s="30"/>
       <c r="J23" s="4"/>
     </row>
-    <row r="24" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:14" ht="25.05" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="3"/>
-      <c r="B24" s="112" t="str">
+      <c r="B24" s="93" t="str">
         <f xml:space="preserve"> _xlfn.CONCAT( Q2, " Cost :")</f>
         <v>Natural Gas Cost :</v>
       </c>
-      <c r="C24" s="113"/>
+      <c r="C24" s="94"/>
       <c r="D24" s="18">
         <f>N19/M19</f>
-        <v>3.278834788077285</v>
+        <v>3.3359863759632882</v>
       </c>
       <c r="E24" s="21" t="s">
         <v>18</v>
@@ -11643,7 +11429,7 @@
       <c r="I24" s="30"/>
       <c r="J24" s="4"/>
     </row>
-    <row r="25" spans="1:14" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:14" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -15288,7 +15074,7 @@
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B21:C21"/>
   </mergeCells>
-  <dataValidations disablePrompts="1" count="2">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2" xr:uid="{9747AF16-8BFF-3245-86C1-E41D734FE8BA}">
       <formula1>$P$7:$P$14</formula1>
     </dataValidation>
@@ -15302,274 +15088,17 @@
   <headerFooter>
     <oddFooter>&amp;L000000Lehigh University IAC&amp;C000000LE0497&amp;R000000Page: &amp;P/</oddFooter>
   </headerFooter>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8D123D0-40E3-422E-BDFC-2CEC98C5B497}">
-  <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="15.86328125" customWidth="1"/>
-    <col min="2" max="2" width="15.59765625" customWidth="1"/>
-    <col min="4" max="4" width="18.86328125" customWidth="1"/>
-    <col min="7" max="7" width="10.1328125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" ht="30.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="93" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="94" t="s">
-        <v>51</v>
-      </c>
-      <c r="C1" s="94" t="s">
-        <v>52</v>
-      </c>
-      <c r="D1" s="94" t="s">
-        <v>53</v>
-      </c>
-      <c r="E1" s="94" t="s">
-        <v>52</v>
-      </c>
-      <c r="F1" s="94" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="94" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="15.4" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="108" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2" s="95" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" s="95" t="s">
-        <v>56</v>
-      </c>
-      <c r="D2" s="95" t="s">
-        <v>55</v>
-      </c>
-      <c r="E2" s="95" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="95" t="s">
-        <v>56</v>
-      </c>
-      <c r="G2" s="95" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="16.149999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="96" t="s">
-        <v>62</v>
-      </c>
-      <c r="B3" s="97">
-        <v>8062000</v>
-      </c>
-      <c r="C3" s="110">
-        <v>6.0000000000000001E-3</v>
-      </c>
-      <c r="D3" s="97">
-        <v>8013000</v>
-      </c>
-      <c r="E3" s="111">
-        <v>6.4999999999999997E-3</v>
-      </c>
-      <c r="F3" s="98">
-        <v>0</v>
-      </c>
-      <c r="G3" s="99">
-        <v>100456.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="96" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="97">
-        <v>10293000</v>
-      </c>
-      <c r="C4" s="110">
-        <v>6.0000000000000001E-3</v>
-      </c>
-      <c r="D4" s="97">
-        <v>11485000</v>
-      </c>
-      <c r="E4" s="111">
-        <v>6.4999999999999997E-3</v>
-      </c>
-      <c r="F4" s="98">
-        <v>0</v>
-      </c>
-      <c r="G4" s="99">
-        <v>136410.5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="96" t="s">
-        <v>60</v>
-      </c>
-      <c r="B5" s="97">
-        <v>10882000</v>
-      </c>
-      <c r="C5" s="110">
-        <v>6.0000000000000001E-3</v>
-      </c>
-      <c r="D5" s="97">
-        <v>8081000</v>
-      </c>
-      <c r="E5" s="111">
-        <v>6.4999999999999997E-3</v>
-      </c>
-      <c r="F5" s="98">
-        <v>0</v>
-      </c>
-      <c r="G5" s="99">
-        <v>117818.5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="96" t="s">
-        <v>61</v>
-      </c>
-      <c r="B6" s="97">
-        <v>7165000</v>
-      </c>
-      <c r="C6" s="110">
-        <v>6.0000000000000001E-3</v>
-      </c>
-      <c r="D6" s="97">
-        <v>5549000</v>
-      </c>
-      <c r="E6" s="111">
-        <v>6.4999999999999997E-3</v>
-      </c>
-      <c r="F6" s="98">
-        <v>0</v>
-      </c>
-      <c r="G6" s="99">
-        <v>79058.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="96"/>
-      <c r="B7" s="97"/>
-      <c r="C7" s="98"/>
-      <c r="D7" s="97"/>
-      <c r="E7" s="98"/>
-      <c r="F7" s="98"/>
-      <c r="G7" s="99"/>
-    </row>
-    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="96"/>
-      <c r="B8" s="97"/>
-      <c r="C8" s="98"/>
-      <c r="D8" s="97"/>
-      <c r="E8" s="98"/>
-      <c r="F8" s="98"/>
-      <c r="G8" s="99"/>
-    </row>
-    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="96"/>
-      <c r="B9" s="97"/>
-      <c r="C9" s="98"/>
-      <c r="D9" s="97"/>
-      <c r="E9" s="98"/>
-      <c r="F9" s="98"/>
-      <c r="G9" s="99"/>
-    </row>
-    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A10" s="96"/>
-      <c r="B10" s="97"/>
-      <c r="C10" s="98"/>
-      <c r="D10" s="97"/>
-      <c r="E10" s="98"/>
-      <c r="F10" s="98"/>
-      <c r="G10" s="99"/>
-    </row>
-    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="96"/>
-      <c r="B11" s="97"/>
-      <c r="C11" s="98"/>
-      <c r="D11" s="97"/>
-      <c r="E11" s="98"/>
-      <c r="F11" s="98"/>
-      <c r="G11" s="99"/>
-    </row>
-    <row r="12" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A12" s="96"/>
-      <c r="B12" s="97"/>
-      <c r="C12" s="98"/>
-      <c r="D12" s="97"/>
-      <c r="E12" s="98"/>
-      <c r="F12" s="98"/>
-      <c r="G12" s="99"/>
-    </row>
-    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A13" s="96"/>
-      <c r="B13" s="97"/>
-      <c r="C13" s="98"/>
-      <c r="D13" s="97"/>
-      <c r="E13" s="98"/>
-      <c r="F13" s="98"/>
-      <c r="G13" s="99"/>
-    </row>
-    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="100"/>
-      <c r="B14" s="101"/>
-      <c r="C14" s="102"/>
-      <c r="D14" s="101"/>
-      <c r="E14" s="102"/>
-      <c r="F14" s="102"/>
-      <c r="G14" s="103"/>
-    </row>
-    <row r="15" spans="1:7" ht="16.149999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="104" t="s">
-        <v>4</v>
-      </c>
-      <c r="B15" s="101"/>
-      <c r="C15" s="102"/>
-      <c r="D15" s="101"/>
-      <c r="E15" s="102"/>
-      <c r="F15" s="102"/>
-      <c r="G15" s="103"/>
-    </row>
-    <row r="16" spans="1:7" ht="16.149999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="104" t="s">
-        <v>57</v>
-      </c>
-      <c r="B16" s="105">
-        <v>6.7000000000000002E-3</v>
-      </c>
-      <c r="C16" s="106" t="s">
-        <v>58</v>
-      </c>
-      <c r="D16" s="105">
-        <v>1.2E-2</v>
-      </c>
-      <c r="E16" s="106" t="s">
-        <v>58</v>
-      </c>
-      <c r="F16" s="107"/>
-      <c r="G16" s="107"/>
-    </row>
-    <row r="17" ht="13.15" thickTop="1" x14ac:dyDescent="0.35"/>
-  </sheetData>
-  <phoneticPr fontId="19" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="U1:U1002"/>
-  <sheetFormatPr defaultColWidth="12.73046875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.73046875" customWidth="1"/>
+    <col min="1" max="1" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="21:21" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -16605,40 +16134,40 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr codeName="Sheet3">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:S990"/>
-  <sheetFormatPr defaultColWidth="12.73046875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="5" width="15.86328125" customWidth="1"/>
-    <col min="6" max="6" width="8.86328125" customWidth="1"/>
-    <col min="7" max="12" width="15.86328125" customWidth="1"/>
-    <col min="13" max="19" width="8.86328125" customWidth="1"/>
+    <col min="1" max="5" width="15.796875" customWidth="1"/>
+    <col min="6" max="6" width="8.796875" customWidth="1"/>
+    <col min="7" max="12" width="15.796875" customWidth="1"/>
+    <col min="13" max="19" width="8.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:19" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="22"/>
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
       <c r="D1" s="22"/>
     </row>
-    <row r="2" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="22"/>
-      <c r="B2" s="128" t="s">
+      <c r="B2" s="109" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="129"/>
-      <c r="D2" s="129"/>
-      <c r="E2" s="130"/>
-    </row>
-    <row r="3" spans="1:19" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="131"/>
-      <c r="C3" s="132"/>
-      <c r="D3" s="132"/>
-      <c r="E3" s="133"/>
+      <c r="C2" s="110"/>
+      <c r="D2" s="110"/>
+      <c r="E2" s="111"/>
+    </row>
+    <row r="3" spans="1:19" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="B3" s="112"/>
+      <c r="C3" s="113"/>
+      <c r="D3" s="113"/>
+      <c r="E3" s="114"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
@@ -16652,7 +16181,7 @@
       <c r="R3" s="2"/>
       <c r="S3" s="2"/>
     </row>
-    <row r="4" spans="1:19" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:19" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B4" s="61" t="s">
         <v>21</v>
       </c>
@@ -16678,21 +16207,21 @@
       <c r="R4" s="2"/>
       <c r="S4" s="2"/>
     </row>
-    <row r="5" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B5" s="27" t="s">
         <v>0</v>
       </c>
       <c r="C5" s="8">
         <f>'Raw Data'!C19</f>
-        <v>66243000</v>
+        <v>12362093</v>
       </c>
       <c r="D5" s="8">
         <f>'Raw Data'!I19</f>
-        <v>684912.47272727266</v>
+        <v>127816.54944242424</v>
       </c>
       <c r="E5" s="9">
         <f>'Raw Data'!D19</f>
-        <v>4472064.93</v>
+        <v>1454221.3599999999</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -16707,7 +16236,7 @@
       <c r="R5" s="2"/>
       <c r="S5" s="2"/>
     </row>
-    <row r="6" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B6" s="28" t="s">
         <v>2</v>
       </c>
@@ -16719,7 +16248,7 @@
       </c>
       <c r="E6" s="31">
         <f>'Raw Data'!F19</f>
-        <v>223589.91</v>
+        <v>148361.25999999998</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -16734,7 +16263,7 @@
       <c r="R6" s="2"/>
       <c r="S6" s="2"/>
     </row>
-    <row r="7" spans="1:19" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:19" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B7" s="64" t="str">
         <f>'Raw Data'!Q2</f>
         <v>Natural Gas</v>
@@ -16744,11 +16273,11 @@
       </c>
       <c r="D7" s="47">
         <f>'Raw Data'!M19</f>
-        <v>201786.07120000003</v>
+        <v>202404.21090000001</v>
       </c>
       <c r="E7" s="48">
         <f>'Raw Data'!N19</f>
-        <v>661623.19000000006</v>
+        <v>675217.69000000006</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -16763,7 +16292,7 @@
       <c r="R7" s="2"/>
       <c r="S7" s="2"/>
     </row>
-    <row r="8" spans="1:19" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:19" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="B8" s="41" t="s">
         <v>4</v>
       </c>
@@ -16772,11 +16301,11 @@
       </c>
       <c r="D8" s="50">
         <f t="shared" ref="D8:E8" si="0">SUM(D5:D7)</f>
-        <v>886698.54392727267</v>
+        <v>330220.76034242427</v>
       </c>
       <c r="E8" s="51">
         <f t="shared" si="0"/>
-        <v>5357278.03</v>
+        <v>2277800.31</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -16791,7 +16320,7 @@
       <c r="R8" s="2"/>
       <c r="S8" s="2"/>
     </row>
-    <row r="9" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -16805,7 +16334,7 @@
       <c r="R9" s="2"/>
       <c r="S9" s="2"/>
     </row>
-    <row r="10" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -16826,7 +16355,7 @@
       <c r="R10" s="2"/>
       <c r="S10" s="2"/>
     </row>
-    <row r="11" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -16847,7 +16376,7 @@
       <c r="R11" s="2"/>
       <c r="S11" s="2"/>
     </row>
-    <row r="12" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -16868,7 +16397,7 @@
       <c r="R12" s="2"/>
       <c r="S12" s="2"/>
     </row>
-    <row r="13" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -16889,7 +16418,7 @@
       <c r="R13" s="2"/>
       <c r="S13" s="2"/>
     </row>
-    <row r="14" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -16910,7 +16439,7 @@
       <c r="R14" s="2"/>
       <c r="S14" s="2"/>
     </row>
-    <row r="15" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -16931,7 +16460,7 @@
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
     </row>
-    <row r="16" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -16952,7 +16481,7 @@
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
     </row>
-    <row r="17" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -16973,7 +16502,7 @@
       <c r="R17" s="2"/>
       <c r="S17" s="2"/>
     </row>
-    <row r="18" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -16994,7 +16523,7 @@
       <c r="R18" s="2"/>
       <c r="S18" s="2"/>
     </row>
-    <row r="19" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -17015,7 +16544,7 @@
       <c r="R19" s="2"/>
       <c r="S19" s="2"/>
     </row>
-    <row r="20" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -17036,7 +16565,7 @@
       <c r="R20" s="2"/>
       <c r="S20" s="2"/>
     </row>
-    <row r="21" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -17057,7 +16586,7 @@
       <c r="R21" s="2"/>
       <c r="S21" s="2"/>
     </row>
-    <row r="22" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -17078,7 +16607,7 @@
       <c r="R22" s="2"/>
       <c r="S22" s="2"/>
     </row>
-    <row r="23" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -17099,7 +16628,7 @@
       <c r="R23" s="2"/>
       <c r="S23" s="2"/>
     </row>
-    <row r="24" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -17120,7 +16649,7 @@
       <c r="R24" s="2"/>
       <c r="S24" s="2"/>
     </row>
-    <row r="25" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -17141,7 +16670,7 @@
       <c r="R25" s="2"/>
       <c r="S25" s="2"/>
     </row>
-    <row r="26" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -17162,7 +16691,7 @@
       <c r="R26" s="2"/>
       <c r="S26" s="2"/>
     </row>
-    <row r="27" spans="1:19" ht="24.95" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:19" ht="25.05" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -21793,34 +21322,34 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0F00-000000000000}">
   <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:H996"/>
-  <sheetFormatPr defaultColWidth="12.73046875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="6" width="15.86328125" style="22" customWidth="1"/>
-    <col min="7" max="14" width="15.86328125" customWidth="1"/>
+    <col min="1" max="6" width="15.796875" style="22" customWidth="1"/>
+    <col min="7" max="14" width="15.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="2" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="B2" s="128" t="s">
+    <row r="1" spans="2:6" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="B2" s="109" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="134"/>
-      <c r="D2" s="134"/>
-      <c r="E2" s="135"/>
+      <c r="C2" s="115"/>
+      <c r="D2" s="115"/>
+      <c r="E2" s="116"/>
       <c r="F2" s="70"/>
     </row>
-    <row r="3" spans="2:6" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="B3" s="136"/>
-      <c r="C3" s="137"/>
-      <c r="D3" s="137"/>
-      <c r="E3" s="138"/>
+    <row r="3" spans="2:6" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="B3" s="117"/>
+      <c r="C3" s="118"/>
+      <c r="D3" s="118"/>
+      <c r="E3" s="119"/>
       <c r="F3" s="70"/>
     </row>
-    <row r="4" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="52" t="s">
         <v>14</v>
       </c>
@@ -21836,7 +21365,7 @@
       </c>
       <c r="F4" s="73"/>
     </row>
-    <row r="5" spans="2:6" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:6" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="55" t="s">
         <v>15</v>
       </c>
@@ -21851,253 +21380,253 @@
       </c>
       <c r="F5" s="73"/>
     </row>
-    <row r="6" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="23" t="str">
         <f>'Raw Data'!B7</f>
-        <v>Oct 23</v>
+        <v>Jan 24</v>
       </c>
       <c r="C6" s="8">
         <f>'Raw Data'!D7</f>
-        <v>336267.31</v>
+        <v>106397.86</v>
       </c>
       <c r="D6" s="8">
         <f>'Raw Data'!F7</f>
-        <v>17843.61</v>
+        <v>3727.2400000000002</v>
       </c>
       <c r="E6" s="9">
         <f>'Raw Data'!N7</f>
-        <v>49724.82</v>
+        <v>87857.74</v>
       </c>
       <c r="F6" s="72"/>
     </row>
-    <row r="7" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="23" t="str">
         <f>'Raw Data'!B8</f>
-        <v>Nov 23</v>
+        <v>Feb 24</v>
       </c>
       <c r="C7" s="8">
         <f>'Raw Data'!D8</f>
-        <v>337009.91999999998</v>
+        <v>95101.49</v>
       </c>
       <c r="D7" s="8">
         <f>'Raw Data'!F8</f>
-        <v>17843.61</v>
+        <v>3654.9300000000003</v>
       </c>
       <c r="E7" s="9">
         <f>'Raw Data'!N8</f>
-        <v>13191.5</v>
+        <v>65523.329999999994</v>
       </c>
       <c r="F7" s="72"/>
     </row>
-    <row r="8" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="23" t="str">
         <f>'Raw Data'!B9</f>
-        <v>Dec 23</v>
+        <v>Mar 24</v>
       </c>
       <c r="C8" s="8">
         <f>'Raw Data'!D9</f>
-        <v>403169.72</v>
+        <v>100800.73</v>
       </c>
       <c r="D8" s="8">
         <f>'Raw Data'!F9</f>
-        <v>20304.8</v>
+        <v>4105.5200000000004</v>
       </c>
       <c r="E8" s="9">
         <f>'Raw Data'!N9</f>
-        <v>43547.51</v>
+        <v>66562.8</v>
       </c>
       <c r="F8" s="72"/>
     </row>
-    <row r="9" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="23" t="str">
         <f>'Raw Data'!B10</f>
-        <v>Jan 24</v>
+        <v>Apr 24</v>
       </c>
       <c r="C9" s="8">
         <f>'Raw Data'!D10</f>
-        <v>431726.45</v>
+        <v>121946.65</v>
       </c>
       <c r="D9" s="8">
         <f>'Raw Data'!F10</f>
-        <v>21535.39</v>
+        <v>4318.84</v>
       </c>
       <c r="E9" s="9">
         <f>'Raw Data'!N10</f>
-        <v>251777.42</v>
+        <v>52165.7</v>
       </c>
       <c r="F9" s="72"/>
     </row>
-    <row r="10" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="23" t="str">
         <f>'Raw Data'!B11</f>
-        <v>Feb 24</v>
+        <v>May 24</v>
       </c>
       <c r="C10" s="8">
         <f>'Raw Data'!D11</f>
-        <v>361043.48</v>
+        <v>117553.12999999999</v>
       </c>
       <c r="D10" s="8">
         <f>'Raw Data'!F11</f>
-        <v>17228.310000000001</v>
+        <v>4585.8</v>
       </c>
       <c r="E10" s="9">
         <f>'Raw Data'!N11</f>
-        <v>58848.990000000005</v>
+        <v>49743.42</v>
       </c>
       <c r="F10" s="72"/>
     </row>
-    <row r="11" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="23" t="str">
         <f>'Raw Data'!B12</f>
-        <v>Mar 24</v>
+        <v>Jun 24</v>
       </c>
       <c r="C11" s="8">
         <f>'Raw Data'!D12</f>
-        <v>383119.25</v>
+        <v>137534.25</v>
       </c>
       <c r="D11" s="8">
         <f>'Raw Data'!F12</f>
-        <v>18458.91</v>
+        <v>26620.42</v>
       </c>
       <c r="E11" s="9">
         <f>'Raw Data'!N12</f>
-        <v>-3183.3199999999997</v>
+        <v>46165.399999999994</v>
       </c>
       <c r="F11" s="72"/>
     </row>
-    <row r="12" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="23" t="str">
         <f>'Raw Data'!B13</f>
-        <v>Apr 24</v>
+        <v>Jul 24</v>
       </c>
       <c r="C12" s="8">
         <f>'Raw Data'!D13</f>
-        <v>394258.4</v>
+        <v>151332.35</v>
       </c>
       <c r="D12" s="8">
         <f>'Raw Data'!F13</f>
-        <v>19689.5</v>
+        <v>29423.26</v>
       </c>
       <c r="E12" s="9">
         <f>'Raw Data'!N13</f>
-        <v>61041.850000000006</v>
+        <v>48984.39</v>
       </c>
       <c r="F12" s="72"/>
     </row>
-    <row r="13" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="23" t="str">
         <f>'Raw Data'!B14</f>
-        <v>May 24</v>
+        <v>Aug 24</v>
       </c>
       <c r="C13" s="8">
         <f>'Raw Data'!D14</f>
-        <v>340182.89</v>
+        <v>141123.71</v>
       </c>
       <c r="D13" s="8">
         <f>'Raw Data'!F14</f>
-        <v>17843.61</v>
+        <v>29498.550000000003</v>
       </c>
       <c r="E13" s="9">
         <f>'Raw Data'!N14</f>
-        <v>42994.85</v>
+        <v>50635.75</v>
       </c>
       <c r="F13" s="72"/>
     </row>
-    <row r="14" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="23" t="str">
         <f>'Raw Data'!B15</f>
-        <v>Jun 24</v>
+        <v>Sep 24</v>
       </c>
       <c r="C14" s="8">
         <f>'Raw Data'!D15</f>
-        <v>359558.26</v>
+        <v>131091.88999999998</v>
       </c>
       <c r="D14" s="8">
         <f>'Raw Data'!F15</f>
-        <v>18271.48</v>
+        <v>26660.23</v>
       </c>
       <c r="E14" s="9">
         <f>'Raw Data'!N15</f>
-        <v>37352.270000000004</v>
+        <v>51575.020000000004</v>
       </c>
       <c r="F14" s="72"/>
     </row>
-    <row r="15" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="23" t="str">
         <f>'Raw Data'!B16</f>
-        <v>Jul 24</v>
+        <v>Oct 24</v>
       </c>
       <c r="C15" s="8">
         <f>'Raw Data'!D16</f>
-        <v>397363.86</v>
+        <v>119489.42</v>
       </c>
       <c r="D15" s="8">
         <f>'Raw Data'!F16</f>
-        <v>19189.689999999999</v>
+        <v>4596.1099999999997</v>
       </c>
       <c r="E15" s="9">
         <f>'Raw Data'!N16</f>
-        <v>35079.659999999996</v>
+        <v>53352.630000000005</v>
       </c>
       <c r="F15" s="72"/>
     </row>
-    <row r="16" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="23" t="str">
         <f>'Raw Data'!B17</f>
-        <v>Aug 24</v>
+        <v>Nov 24</v>
       </c>
       <c r="C16" s="8">
         <f>'Raw Data'!D17</f>
-        <v>376165.72</v>
+        <v>115818.54000000001</v>
       </c>
       <c r="D16" s="8">
         <f>'Raw Data'!F17</f>
-        <v>17390.66</v>
+        <v>6038.83</v>
       </c>
       <c r="E16" s="9">
         <f>'Raw Data'!N17</f>
-        <v>34223.160000000003</v>
+        <v>75418.23</v>
       </c>
       <c r="F16" s="72"/>
     </row>
-    <row r="17" spans="2:6" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:6" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B17" s="40" t="str">
         <f>'Raw Data'!B18</f>
-        <v>Sep 24</v>
+        <v>Dec 24</v>
       </c>
       <c r="C17" s="47">
         <f>'Raw Data'!D18</f>
-        <v>352199.67</v>
+        <v>116031.34</v>
       </c>
       <c r="D17" s="47">
         <f>'Raw Data'!F18</f>
-        <v>17990.34</v>
+        <v>5131.53</v>
       </c>
       <c r="E17" s="48">
         <f>'Raw Data'!N18</f>
-        <v>37024.480000000003</v>
+        <v>27233.280000000002</v>
       </c>
       <c r="F17" s="72"/>
     </row>
-    <row r="18" spans="2:6" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:6" ht="25.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B18" s="58" t="s">
         <v>4</v>
       </c>
       <c r="C18" s="59">
         <f>'Raw Data'!D19</f>
-        <v>4472064.93</v>
+        <v>1454221.3599999999</v>
       </c>
       <c r="D18" s="59">
         <f>'Raw Data'!F19</f>
-        <v>223589.91</v>
+        <v>148361.25999999998</v>
       </c>
       <c r="E18" s="60">
         <f>'Raw Data'!N19</f>
-        <v>661623.19000000006</v>
+        <v>675217.69000000006</v>
       </c>
       <c r="F18" s="72"/>
     </row>
-    <row r="19" spans="2:6" ht="24.95" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="19" spans="2:6" ht="25.05" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="20" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="21" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="22" spans="2:6" ht="12.75" customHeight="1" x14ac:dyDescent="0.35"/>

</xml_diff>